<commit_message>
deploy: refresh downloadable workbook
</commit_message>
<xml_diff>
--- a/AutoCava_AI最新统计表.xlsx
+++ b/AutoCava_AI最新统计表.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并数据表" sheetId="1" r:id="R295a71fde0c64aec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径说明" sheetId="2" r:id="R7ac048be70634af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并数据表" sheetId="1" r:id="R5c192cadf0f34090"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径说明" sheetId="2" r:id="Rc0c23b8f58a04469"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
deploy: dashboard 08/17-08/30 (direct-read caliber, JSON realigned)
</commit_message>
<xml_diff>
--- a/AutoCava_AI最新统计表.xlsx
+++ b/AutoCava_AI最新统计表.xlsx
@@ -749,22 +749,22 @@
         <v>1.460089</v>
       </c>
       <c r="C5" s="6">
-        <v>1.525641</v>
+        <v>1.5452436194895591</v>
       </c>
       <c r="D5" s="6">
-        <v>1.4892086330935252</v>
+        <v>1.4705882352941178</v>
       </c>
       <c r="E5" s="6">
-        <v>1.5254237288135593</v>
+        <v>1.5816326530612246</v>
       </c>
       <c r="F5" s="6">
-        <v>1.633969118982743</v>
+        <v>1.624</v>
       </c>
       <c r="G5" s="6">
-        <v>1.5922421948912016</v>
+        <v>1.5313152400835073</v>
       </c>
       <c r="H5" s="6">
-        <v>1.58227</v>
+        <v>1.5749525616698292</v>
       </c>
       <c r="I5" s="6">
         <v>1.4867060561299852</v>
@@ -796,22 +796,22 @@
         <v>205</v>
       </c>
       <c r="C6" s="4">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D6" s="4">
-        <v>226</v>
+        <v>204</v>
       </c>
       <c r="E6" s="4">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="F6" s="4">
-        <v>293</v>
+        <v>322</v>
       </c>
       <c r="G6" s="4">
-        <v>277</v>
+        <v>236</v>
       </c>
       <c r="H6" s="4">
-        <v>342</v>
+        <v>391</v>
       </c>
       <c r="I6" s="4">
         <v>319</v>
@@ -843,22 +843,22 @@
         <v>0.22503</v>
       </c>
       <c r="C7" s="5">
-        <v>0.26866</v>
+        <v>0.2675086107921929</v>
       </c>
       <c r="D7" s="5">
-        <v>0.2857142857142857</v>
+        <v>0.2579013906447535</v>
       </c>
       <c r="E7" s="5">
-        <v>0.25435540069686413</v>
+        <v>0.2659698025551684</v>
       </c>
       <c r="F7" s="5">
-        <v>0.24016393442622952</v>
+        <v>0.2639344262295082</v>
       </c>
       <c r="G7" s="5">
-        <v>0.29499467518636846</v>
+        <v>0.25133120340788073</v>
       </c>
       <c r="H7" s="5">
-        <v>0.21909</v>
+        <v>0.2504804612427931</v>
       </c>
       <c r="I7" s="5">
         <v>0.2396694214876033</v>

</xml_diff>